<commit_message>
up to date processor
</commit_message>
<xml_diff>
--- a/src/cubes/data/energy_systems/batteries.xlsx
+++ b/src/cubes/data/energy_systems/batteries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottjeen/phd/research/CUBES/src/cubes/data/energy_systems/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6018C651-FC78-FE40-8A82-E64FB353B3BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815CD103-7755-D648-910F-1C1D1240F0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2060" yWindow="2880" windowWidth="26840" windowHeight="15940" xr2:uid="{044ACA5D-B511-514B-9BD5-CA53B5FB19D2}"/>
   </bookViews>
@@ -68,13 +68,13 @@
     <t>https://uk.ecoflow.com/pages/smart-home-ecosystem?utm_source=google&amp;utm_medium=display&amp;utm_campaign=Alwayson&amp;gad=1&amp;gclid=CjwKCAjwxr2iBhBJEiwAdXECwxNzuoIYoVag1tHactE1EnOeKuyeTAz4g2o5rXhbh_H4s59h9Iq8RxoCB8kQAvD_BwE</t>
   </si>
   <si>
-    <t xml:space="preserve">SMALL BATTERY SIZE PROBABILITY  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEDIUM BATTERY SIZE PROBABILITY  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">LARGE BATTERY SIZE PROBABILITY  </t>
+    <t>SMALL BATTERY SIZE PROBABILITY</t>
+  </si>
+  <si>
+    <t>MEDIUM BATTERY SIZE PROBABILITY</t>
+  </si>
+  <si>
+    <t>LARGE BATTERY SIZE PROBABILITY</t>
   </si>
 </sst>
 </file>
@@ -82,7 +82,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -125,7 +125,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -671,5 +671,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>